<commit_message>
feat: done tieu chi import
</commit_message>
<xml_diff>
--- a/src/main/resources/qm/public/resources/qualityCriteriaImportSchema_en.xlsx
+++ b/src/main/resources/qm/public/resources/qualityCriteriaImportSchema_en.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dungn\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\qcadoo_demo\mes\mes-plugins\fti-plugins-qm\src\main\resources\qm\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3EE6111D-A44E-4104-9C62-0F3CD67EDC28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E43B4187-58CF-4739-A223-7EF072506750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4005ADB-0ECA-4B65-AC63-34404DD8E1BE}"/>
   </bookViews>
@@ -437,6 +437,14 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1:D1048576" xr:uid="{F2C2884E-DA38-4044-9170-472878A5CABA}">
+      <formula1>"cm, cm2, dam, dm, g, hl, kg, l, m, m2, m3, mm, Nm, pack, pair, pc, set, tank, Y/N"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C1048576" xr:uid="{735AC447-7A61-4D3C-9017-F51B567BC293}">
+      <formula1>"Qualitative, Quantitative"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>